<commit_message>
fix anu gendeng pelahap ram
</commit_message>
<xml_diff>
--- a/P8/scraping/hasil_cleaning.xlsx
+++ b/P8/scraping/hasil_cleaning.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,35 +460,140 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Meta Rilis Kacamata Pintar Murah, Siap Gantikan Smartphone?</t>
+          <t>Quote Jack Ma buat Rakyat Kecil, Dia Sendiri jadi Buktinya</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Meta Rilis Kacamata Pintar Murah, Siap Gantikan Smartphone?</t>
+          <t>Quote Jack Ma buat Rakyat Kecil, Dia Sendiri jadi Buktinya</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8546207/meta-rilis-kacamata-pintar-murah-siap-gantikan-smartphone</t>
+          <t>https://inet.detik.com/cyberlife/d-8550306/quote-jack-ma-buat-rakyat-kecil-dia-sendiri-jadi-buktinya</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8546207/meta-rilis-kacamata-pintar-murah-siap-gantikan-smartphone</t>
+          <t>https://inet.detik.com/cyberlife/d-8550306/quote-jack-ma-buat-rakyat-kecil-dia-sendiri-jadi-buktinya</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/24/meta-glasses-1782306203775_43.webp?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2023/01/03/jack-ma_43.png?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>46198.39799424111</v>
+        <v>46201.36687434572</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Jakarta - Meta mengumumkan seri kacamata pintar baru seharga USD 299, yang setidaknya USD 80 lebih murah dari kacamata Meta Ray Ban generasi kedua kelas entry level. CEO Mark Zuckerberg tampaknya kian gencar berekspansi ke ranah perangkat wearable. Meta Glasses ini hadir dengan desain baru dan diproduksi melalui kerja sama dengan EssilorLuxottica, perusahaan induk Ray-Ban. Namun dikutip detikINET dari CNBC, kacamata ini tak lagi mengusung merek Ray-Ban maupun Oakley. Meta memasarkan kacamata pintarnya secara agresif terkait memanasnya persaingan dan meningkatnya minat konsumen terhadap perangkat augmented reality. Meski pasar kacamata pintar masih tergolong kecil, Meta dan EssilorLuxottica berhasil mendominasi dengan perkiraan pangsa pasar melampaui 80%, serta mencatatkan jutaan unit terjual sejak peluncuran perdana tahun 2021. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca juga: Diklaim Calon Pengganti Smartphone, Gadget Ini Tuai Kritik Meta Glasses tidak dilengkapi layar, tapi ada kamera dan speaker terintegrasi. Pengguna dapat berbicara dengan AI Meta untuk menerjemahkan atau memahami apa yang mereka lihat di sekelilingnya, serta mengambil foto maupun merekam video dari sekitar. Para eksekutif Meta menyebut kacamata pintar ringan ini batu loncatan menuju perangkat yang lebih mutakhir, yang nantinya akan mengusung layar berlensa dengan kemampuan komputasi. Sebagai informasi, tahun lalu Meta sempat mengumumkan kacamata Ray-Ban Display seharga USD 799 yang sudah dilengkapi layar internal. Zuckerberg tampaknya meraih sukses melalui kacamata pintar dibanding headset virtual reality (VR), perangkat yang sebelumnya jadi alasan perubahan nama Facebook menjadi Meta pada tahun 2021. Pasar VR sejauh ini masih tersegmentasi dan lebih menyasar gamer, sementara Zuck kini fokus menguasai platform hardware di era AI. Visi Zuckerberg: Kacamata Pintar Pengganti Smartphone Sebelumnya, Zuckerberg sempat melontarkan sejumlah pernyataan menarik terkait rencana Meta di kacamata pintar. Ia tampak yakin gadget ini suatu hari nanti akan menggantikan peran smartphone. Ia menegaskan Meta memandang kacamata pintar dan AI berkaitan erat dan merupakan masa depan komputasi. "Kacamata adalah wujud perangkat ideal untuk AI maupun Metaverse. Perangkat ini memungkinkan Anda membiarkan AI melihat apa yang Anda lihat, mendengar apa yang Anda dengar, dan bicara dengan Anda sepanjang hari. Selain itu, kacamata ini memungkinkan Anda memadukan dunia fisik dan digital secara bersamaan melalui wujud hologram," sebut Zuck beberapa waktu silam. "Saat ini, lebih dari satu miliar orang di seluruh dunia memakai kacamata, dan sangat besar kemungkinannya kacamata-kacamata tersebut akan beralih menjadi kacamata AI dalam 5 hingga 10 tahun ke depan," demikian prediksinya. Sementara itu, kompetisi kacamata pintar memanas. Bulan lalu, Google menyatakan sedang mengembangkan kacamata pintar baru bermitra dengan Warby Parker, di mana perangkat tersebut akan ditenagai AI Gemini. Pekan lalu, Snap mengumumkan Specs, kacamata pintar seharga USD 2.195 yang diposisikan oleh CEO Evan Spiegel sebagai penerus smartphone. Baca juga: Para Pentolan Teknologi Ramal Kematian Smartphone Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? (fyk/afr) TAGS meta kacamata pintar mark zuckerberg LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Jack Ma orang biasa yang bertransformasi menjadi salah satu yang paling sukses di China, bahkan dunia. Sebelum menjadi sebesar sekarang, Jack Ma adalah orang yang mengalami kegagalan berulang kali. Laki-laki bernama Ma Yun ini lahir di Hangzhou, China pada tahun 1964. Dia pernah gagal ujian masuk universitas dua kali, setelahnya pun dia ditolak dari 30 lebih kerjaan termasuk di KFC. Tapi bayangkan jika Ma menyerah, tidak akan ada yang namanya eCommerce Alibaba di dunia. Sumbangsihnya untuk edukasi dan amal juga tidak bakal ada. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Jack Ma Sebut Penyebab 99,9% Orang Tidak Punya Masa Depan ADVERTISEMENT Menyadari bahwa dia bukan orang yang punya bekal sejak awal merintis karier, Ma sempat memberikan sebuah quote yang membuat orang terenyuh. Katanya begini: "Ketika Anda kecil, Anda harus sangat fokus dan bergantung pada otak Anda, bukan kekuatan Anda." Tantangan hidup tidak selalu dimenangkan oleh mereka yang memiliki kekuasaan atau sumber daya paling banyak. Terkadang, pemenang sejati tidak lahir dengan keuntungan apa-apa. Tidak uang, tidak pula kekuasaan. Meskipun perjalanan hidup seringkali terasa seperti perlombaan besar di mana yang kuat dan kaya melaju di depan, siapa saja bisa memulai dari kecil. Sekalipun sarana, pengalaman, atau dukungannya terbatas, namun kekuatan sejati berasal dari fokus yang tajam dan pemikiran yang cerdas, bukan kekayaan atau kekuasaan. Jadi, walaupun realistisnya, dunia saat ini menghargai peningkatan karier yang cepat dan kemenangan besar, sebuah nasihat dari salah satu pengusaha dan pendiri sukses ini juga ada benarnya. Ia sendiri membuktikannya karena ia juga memulai semuanya dari nol. Demikian melansir Times of India , Minggu (28/6/2026). Baca Juga : Apa yang Lebih Penting dari Alibaba bagi Jack Ma? Jawabannya Bikin Kagum Mensos RI: "Ayo Jihad Data" Mensos RI: "Ayo Jihad Data" (ask/ask) TAGS jack ma inspirasi motivasi ecommerce LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Antara Rasa Bersalah dan Bertahan Hidup: Dilema Warga Eropa Pakai AC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Antara Rasa Bersalah dan Bertahan Hidup: Dilema Warga Eropa Pakai AC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/science/d-8550304/antara-rasa-bersalah-dan-bertahan-hidup-dilema-warga-eropa-pakai-ac</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/science/d-8550304/antara-rasa-bersalah-dan-bertahan-hidup-dilema-warga-eropa-pakai-ac</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/07/29/ilustrasi-ac-1753768188217_43.jpeg?w=250&amp;q=90</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>46201.36687434572</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Jakarta - Banyak orang Eropa sejak lama menganggap AC sebagai kemewahan tidak perlu, mahal, dan penyumbang emisi karbon. Namun, seiring musim panas di benua itu yang semakin panas dan merenggut korban, pandangan mulai berubah. Sepekan terakhir, 40 orang tewas tenggelam di Prancis saat mencari tempat berendam. Di Spanyol, suhu mencapai sekitar 44 derajat C, dan Inggris menghadapi bulan Juni terpanas. Setiap tahun menurut WHO, cuaca panas merenggut rata-rata 175.000 nyawa di Eropa. Penggunaan AC dapat memangkas tingkat kematian akibat panas hingga 75%, menurut studi tahun 2007. Riset The Lancet menemukan di 2019, 195.000 kematian terkait cuaca panas pada kelompok lansia di atas 65 tahun berhasil dicegah berkat adopsi AC. Namun hanya sekitar 20% orang Eropa memiliki AC di rumah, berbanding 90% di Amerika Serikat. SCROLL TO CONTINUE WITH CONTENT Baca juga: Kepanasan, Warga Eropa Menyerah dan Berbondong Beli AC Budaya, Biaya, dan Iklim Sebagian dari keengganan warga Eropa untuk memasang AC mungkin berasal dari sikap stoikisme historis mereka. Karena AC tidak pernah digunakan pada masa lalu, tidak seharusnya dibutuhkan sekarang. Sebagian besar wilayah Eropa, setidaknya hingga beberapa dekade terakhir, memang tak benar-benar butuh AC. Faktor biaya juga menjadi penghalang. Minimnya pasokan gas alam domestik di banyak negara Eropa mengharuskan mereka mengimpornya, membuat biaya energi di Eropa lebih tinggi dengan gaji lebih rendah dari AS. ADVERTISEMENT Banyak warga Eropa juga dihantui rasa bersalah terhadap dampak iklim penggunaan AC. Penggunaan AC menyumbang 4% total emisi gas rumah kaca global, dua kali lipat industri penerbangan. Sekarang, musim panas di wilayah selatan jadi ekstrem sehingga trik arsitektur tradisional yang digunakan berabad-abad tak mempan. Sementara di utara, rumah yang didesain menahan udara panas agar penghuninya tidak kedinginan, berubah bak "tungku pembakaran" saat musim panas. Di Italia, ribuan kematian selama gelombang panas tahun 2003 jadi titik puncak kesabaran. Musim panas tahun itu, diperkirakan hanya 10-15% rumah tangga punya AC. Namun di 2024, angkanya meroket menjadi 56%. Italia kini menyumbang sepertiga seluruh penggunaan listrik untuk AC di Eropa. Di Prancis, yang minggu ini mengalami hari-hari terpanas, toko-toko mulai kehabisan AC. Di Inggris, sekitar empat juta rumah kini memiliki AC, dua kali lipat dibanding tiga tahun lalu. Bagi Katie di London, memasang AC tidak pernah terlintas, baik karena biaya mahal maupun dampak lingkungan. "Biasanya Anda hanya akan terkapar lemas di sofa dan sekadar mencoba bertahan hidup," katanya. Namun, pandangan itu berubah. Ia dan pasangannya memutuskan membeli AC setelah punya anak. "Rasa bersalah terhadap iklim yang saya rasakan tidak ada apa-apanya dibanding prioritas untuk memastikan bayi saya memiliki tempat tidur aman. Siapa pun yang pernah terjebak selama sejam bagai di neraka, bercucuran keringat sambil mencoba menidurkan bayinya, pasti akan langsung membeli AC, percayalah," katanya. Guna mencegah tren perluasan penggunaan AC ini semakin memperburuk perubahan iklim, pakar menekankan pentingnya pemasangan AC modern yang efisien listrik, ditenagai energi terbarukan seperti tenaga surya. Uni Eropa sendiri berambisi menjadi kawasan netral iklim pada tahun 2050. Guna mewujudkannya, negara-negara seperti Spanyol, Italia, dan Yunani mulai membatasi sejauh mana batas pendinginan ruangan diizinkan di gedung publik selama musim panas. Masyarakat pun disarankan menggabungkan dua solusi, yakni mengombinasikan AC bertenaga surya dengan langkah old school ala masyarakat kawasan Eropa selatan. Baca juga: Ilmuwan Tunjuk Penyebab Suhu Panas Mematikan di Eropa Video: Upgrade AC di Transmart Full Day Sale Aja, Diskonnya Gak Main-main! Video: Upgrade AC di Transmart Full Day Sale Aja, Diskonnya Gak Main-main! (fyk/fyk) TAGS ac eropa gelombang panas LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NASA Temukan Dua Planet Raksasa yang Ringan Seperti Permen Kapas</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NASA Temukan Dua Planet Raksasa yang Ringan Seperti Permen Kapas</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/science/d-8550143/nasa-temukan-dua-planet-raksasa-yang-ringan-seperti-permen-kapas</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/science/d-8550143/nasa-temukan-dua-planet-raksasa-yang-ringan-seperti-permen-kapas</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/26/perbandingan-ukuran-planet-toi-791b-dan-tpi-791c-dengan-planet-di-tata-surya-1782478000277_43.jpeg?w=250&amp;q=90</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>46201.36687434572</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Jakarta - Satelit survei exoplanet (TESS) milik NASA menemukan dua planet 'super mengembang' berukuran raksasa. Walau ukurannya sebesar Jupiter, dua planet ini sangat ringan dengan kepadatan sangat rendah yang sebanding dengan permen kapas. Dua planet tersebut diketahui mengelilingi bintang mirip matahari bernama TOI-791 yang berjarak 1.113 tahun cahaya dari Bumi. TESS pertama kali mendeteksi dua planet ini dengan mengamati penurunan kecerahan TOI-791 yang berulang, tanda bahwa ada planet yang sedang transit dan melewati sebuah bintang. Salah satu planet, yang dinamai TOI-791b, memiliki ukuran yang sama seperti Jupiter, tapi massanya hanya 3% dari planet gas raksasa tersebut. Sementara itu, planet kedua yang disebut TOI-791c bahkan berukuran lebih besar dibanding Jupiter, tapi hanya memiliki 5,9% dari total massanya. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Ilmuwan Ungkap Misteri di Balik Planet Pink yang Unik Kepadatan yang sangat rendah bukan satu-satunya karakteristik luar biasa kedua planet ini. NASA menemukan kedua planet ini terkunci dalam pola orbit yang memungkinkan keduanya dapat saling tarik menarik. Saat mengorbit bintang induknya, dua planet itu bergantian saling menarik, yang mempengaruhi waktu transit mereka saat melintasi bintang induknya. Ilmuwan menggunakan variasi waktu orbit tersebut untuk menghitung massa planet, dan memperkuat status TOI-791b dan TOI-791c sebagai planet dengan kepadatan paling rendah. ADVERTISEMENT "Hanya sedikit dari planet super mengembang ini yang diketahui, dan lebih jarang lagi menemukan dua planet dengan karakteristik ini dalam sistem yang sama," kata kepala tim peneliti George Dransfield dari Universitas Oxford, seperti dikutip dari Space.com, Minggu (28/6/2026). "Kepadatan mereka yang sangat rendah menjadikan mereka target yang menarik untuk memahami bagaimana sistem planet terbentuk dan berevolusi," sambungnya. Baca Juga : Dipimpin Eks Bos Google, Relativity Space Garap Misi Aeolus NASA ke Mars Kedua planet ini juga memiliki waktu orbit yang sangat lama. TOI-791b membutuhkan 139 hari untuk mengelilingi bintangnya, sedangkan TOI-791c membutuhkan 232 hari. Meski begitu, masih banyak hal yang belum diketahui ilmuwan tentang TOI-79b dan TOI 791-c. Dengan observasi lebih lanjut, peneliti berharap dapat mengetahui lebih banyak tentang susunan kimia atmosfernya, bagaimana putarannya mempengaruhi bentuknya, dan bagaimana planet 'permen kapas' seperti itu bisa terbentuk. Video: Bikin Bangga! Siswa SMA di Pinrang Dapat Penghargaan dari NASA Video: Bikin Bangga! Siswa SMA di Pinrang Dapat Penghargaan dari NASA (vmp/vmp) TAGS nasa planet exoplanet LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Kisah Burung Beracun Ditemukan di Papua, Dagingnya 'Membakar'</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kisah Burung Beracun Ditemukan di Papua, Dagingnya 'Membakar'</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/science/d-8550138/kisah-burung-beracun-ditemukan-di-papua-dagingnya-membakar</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/science/d-8550138/kisah-burung-beracun-ditemukan-di-papua-dagingnya-membakar</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/27/burung-beracun-1782555497576_43.webp?w=250&amp;q=90</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46201.36687434572</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Jakarta - Pada tahun 2023, dua spesies burung beracun baru ditemukan dalam ekspedisi ke hutan hujan Papua. Ilmuwan menemukannya dalam penjelajahan ke wilayah tersebut, di mana mereka mengumpulkan sampel dari burung-burung yang memiliki cukup banyak neurotoksin pada bulunya. Spesies terbaru yang masuk dalam daftar burung beracun ini adalah regent whistler (Pachycephala schlegelii) dan rufous-naped bellbird (Aleadryas rufinucha). Burung-burung ini sebenarnya umum ditemukan di wilayah tersebut, namun baru dalam penelitian ini diketahui mereka beracun. Dikutip detikINET dari IFL Science, sudah lebih dari dua dekade sejak spesies burung beracun terakhir ditemukan sehingga penemuan dua spesies beracun ini cukup menghebohkan. SCROLL TO CONTINUE WITH CONTENT Burung-burung ini dipersenjatai Batrachotoxin, berasal dari bahasa Yunani untuk katak (Batrachos). Sebagai salah satu neurotoksin terkuat yang diketahui sains, zat ini dinamai berdasarkan katak panah beracun, tempat racun pertama kali ditemukan. Namun, terbukti zat ini juga terdapat pada spesies non amfibi. Baca juga: Burung Paling Misterius di Indonesia Ditemukan, Bikin Terharu Diyakini bahwa burung-burung tersebut memperoleh toksin melalui pola makan mereka dengan mengonsumsi makanan beracun, yang kemudian diubah menjadi racun dan menyatu ke dalam jaringan tubuh. ADVERTISEMENT Konsentrasi tinggi Batrachotoxin dapat berakibat fatal bagi manusia karena memicu kejang hebat dan akhirnya menyebabkan kematian. Pada kulit katak panah beracun, konsentrasinya cukup untuk menyebabkan gejala parah tersebut, namun pada bulu burung-burung ini dosisnya lebih rendah. Kadar racun tersebut berfungsi sebagai mekanisme pertahanan diri, walau tujuan pastinya belum diketahui pasti. Menurut penduduk setempat, daging burung ini terasa membakar seperti cabai, dan memegang burung ini bukan pengalaman menyenangkan. Ini mengindikasikan mereka beradaptasi agar tidak menarik pemangsa. Dengan bertambahnya spesies burung beracun yang dapat dipelajari, para peneliti bertugas mencari tahu bagaimana dan mengapa mereka menggunakan neurotoksin tersebut. Namun, kerja fisik dalam penelitian ini bisa menyakitkan. "Knud dari Museum Sejarah Alam Denmark mengira saya sedih dan mengalami masa sulit dalam perjalanan itu ketika dia menemukan saya dengan hidung meler dan air mata berlinang. Padahal, saya hanya sedang duduk di sana mengambil sampel bulu seekor Pitohui, salah satu burung paling beracun," kata peneliti University of Copenhagen, Kasun Bodawatta. Proses yang sangat dekat dan personal itulah yang benar-benar menyiksa. "Melepas burung dari jaring tidaklah buruk, tapi ketika sampel harus diambil di lingkungan yang tertutup, Anda bisa merasakan sesuatu di mata dan hidung. Rasanya sedikit seperti mengiris bawang," kisahnya. Baca juga: Berapa Lama Burung Bisa Terbang Tanpa Mendarat? Jawabannya di Luar Nurul Video IPI Sebut Penyerangan Pilot Bisa Putus Distribusi Kebutuhan Warga Papua Video IPI Sebut Penyerangan Pilot Bisa Putus Distribusi Kebutuhan Warga Papua (fyk/fyk) TAGS burung beracun papua LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>

</xml_diff>